<commit_message>
feat: Türkiye Prime Time (3 Shorts / Gün Aşırı 2 Shorts + 1 Uzun) & video_20 başlangıç kilidi
</commit_message>
<xml_diff>
--- a/baslik.xlsx
+++ b/baslik.xlsx
@@ -49,7 +49,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,12 @@
         <bgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border/>
@@ -86,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -128,6 +134,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1897,47 +1909,47 @@
       <c r="AC20" s="6" t="n"/>
     </row>
     <row r="21" ht="112.5" customHeight="1" s="13">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>BEKLEMEDE</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>video_17.mp4</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>Everest'in 2.5 Katı Yüksekliğinde Bir Dağ Var — Ama Dünya'da Değil! 🌋🪐 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>Mars'taki Olympus Mons, yaklaşık 22 km yüksekliğiyle Everest'in 2.5 katı! Tabanı ise Arizona kadar geniş. Dünya'da bu dağın ağırlığı kendi kabuğunu çökerterek batmasına neden olurdu — Mars'ta kabuk buna izin veriyor!</t>
         </is>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>bilgidozu, mars, olympusmons, uzay, geoloji, bilim, shorts</t>
         </is>
       </c>
-      <c r="G21" s="14" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>Olympus Mons'un zirvesinden manzara... 🌋 Peki tırmanır mıydın? Korkanlar 1, cesurlar 2! 👇</t>
         </is>
       </c>
-      <c r="H21" s="14" t="inlineStr">
+      <c r="H21" s="16" t="inlineStr">
         <is>
           <t>Uzay ve Astronomi</t>
         </is>
       </c>
-      <c r="I21" s="14" t="inlineStr">
+      <c r="I21" s="16" t="inlineStr">
         <is>
           <t>NASA — Mars Facts: https://science.nasa.gov/mars/facts/</t>
         </is>
@@ -1964,47 +1976,47 @@
       <c r="AC21" s="6" t="n"/>
     </row>
     <row r="22" ht="112.5" customHeight="1" s="13">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BEKLEMEDE </t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>video_18.mp4</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>Bu Hayvanın BEYNİ YOK — Ama Görüyor, Hissediyor! ⭐🌊 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Denizyıldızının merkezî bir beyni yok: sinir sistemi kollarına yayılmış! Her kolun ucundaki minik gözcükler ışığı algılar, binlerce ayakçık tadar, kavrar ve yürür. Kafasız ama eksiksiz — doğanın en zarif dağıtık zekâ tasarımı!</t>
         </is>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>bilgidozu, denizyıldızı, denizcanlıları, biyoloji, ilginçbilgiler, shorts</t>
         </is>
       </c>
-      <c r="G22" s="14" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
         <is>
           <t>Beyinsiz ama görüyor, tadıyor, yürüyor... ⭐ Doğanın en garip tasarımı mı? 1 yazsın! 👇</t>
         </is>
       </c>
-      <c r="H22" s="14" t="inlineStr">
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>Doğa ve Hayvanlar</t>
         </is>
       </c>
-      <c r="I22" s="14" t="inlineStr">
+      <c r="I22" s="16" t="inlineStr">
         <is>
           <t>Starfish: https://en.wikipedia.org/wiki/Starfish</t>
         </is>
@@ -2031,47 +2043,47 @@
       <c r="AC22" s="6" t="n"/>
     </row>
     <row r="23" ht="112.5" customHeight="1" s="13">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>BEKLEMEDE</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>video_19.mp4</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
         <is>
           <t>Yunuslar Tek Gözü Açık Uyur! 🐬😴 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>Yunusun beyninin iki yarısı sırayla uyur: bir yarı derin uykudayken diğeri düşman nöbeti tutar, yüzer ve nefes aldırır! Göz de beynin uyuyan tarafına göre kapanır. Adı: yarım küre uykusu (USWS) — doğanın nöbetçi sistemi!</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #doğa #bilim</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>bilgidozu, yunus, hayvanlaralemi, uyku, deniz, bilim, shorts</t>
         </is>
       </c>
-      <c r="G23" s="14" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr">
         <is>
           <t>Yunus bile nöbet tutarak uyurken sen nasıl uyuyorsun? 😄🐬 Uykucular 1 yazsın!</t>
         </is>
       </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="H23" s="16" t="inlineStr">
         <is>
           <t>Doğa ve Hayvanlar</t>
         </is>
       </c>
-      <c r="I23" s="14" t="inlineStr">
+      <c r="I23" s="16" t="inlineStr">
         <is>
           <t>Sleep Foundation — Animals and Sleep: https://www.sleepfoundation.org/animals-and-sleep</t>
         </is>

</xml_diff>

<commit_message>
chore(kartal-ai): sync video_33.mp4 (21:24 TR) into status_report.json and workbook
</commit_message>
<xml_diff>
--- a/baslik.xlsx
+++ b/baslik.xlsx
@@ -530,7 +530,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AC112"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" style="13" min="1" max="1"/>
     <col width="22.86" customWidth="1" style="13" min="2" max="2"/>
@@ -3504,54 +3504,62 @@
       <c r="AC39" s="6" t="n"/>
     </row>
     <row r="40" ht="112.5" customHeight="1" s="13">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BEKLEMEDE </t>
-        </is>
-      </c>
-      <c r="B40" s="14" t="inlineStr">
+      <c r="A40" s="19" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
         <is>
           <t>video_33.mp4</t>
         </is>
       </c>
-      <c r="C40" s="14" t="inlineStr">
+      <c r="C40" s="16" t="inlineStr">
         <is>
           <t>Kendini Neden Gıdıklayamazsın? Beynin Hamleni Önceden Biliyor! 🧠🤭 #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D40" s="14" t="inlineStr">
+      <c r="D40" s="16" t="inlineStr">
         <is>
           <t>Başka biri dokunduğunda kolayca gıdıklanırken kendi kendini gıdıklayamamanın sebebi beyinciktir! Beyincik, kendi el hareketini saliseler öncesinden tahmin ederek duyusal kortekse 'bu tehdit değil, kendi dokunuşun' sinyali gönderir ve gıdıklanma tepkisini otomatik olarak bastırır.
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E40" s="14" t="inlineStr">
+      <c r="E40" s="16" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #beyin #psikoloji</t>
         </is>
       </c>
-      <c r="F40" s="14" t="inlineStr">
+      <c r="F40" s="16" t="inlineStr">
         <is>
           <t>bilgidozu, gıdıklanma, beyin, beyincik, nörobilim, psikoloji, ilginçbilgiler, bilim, shorts</t>
         </is>
       </c>
-      <c r="G40" s="14" t="inlineStr">
+      <c r="G40" s="16" t="inlineStr">
         <is>
           <t>Biri dokununca çok gıdıklananlardan mısın? 😄🤭 Evet diyenler '1', bana işlemez diyenler '2' yazsın! 👇</t>
         </is>
       </c>
-      <c r="H40" s="14" t="inlineStr">
+      <c r="H40" s="16" t="inlineStr">
         <is>
           <t>Beyin ve Psikoloji</t>
         </is>
       </c>
-      <c r="I40" s="14" t="inlineStr">
+      <c r="I40" s="16" t="inlineStr">
         <is>
           <t>Wikipedia — Tickling (Self-tickling): https://en.wikipedia.org/wiki/Tickling</t>
         </is>
       </c>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="5" t="n"/>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>https://youtu.be/sh9zYFybcHY</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23 21:24</t>
+        </is>
+      </c>
       <c r="L40" s="5" t="n"/>
       <c r="M40" s="6" t="n"/>
       <c r="N40" s="6" t="n"/>
@@ -8414,6 +8422,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8429,136 +8438,136 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>İşçi Adı</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>Durum</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="0" t="inlineStr">
         <is>
           <t>Son Güncelleme Zamanı</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="0" t="inlineStr">
         <is>
           <t>Son Hata Mesajı</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="0" t="inlineStr">
         <is>
           <t>Kaç İş Yaptı</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="0" t="inlineStr">
         <is>
           <t>Son İşlem Özeti</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>Yükleyici (Drive -&gt; YouTube)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>Çalışıyor</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>2026-10-23 18:29</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="n">
+      <c r="D2" s="0" t="inlineStr"/>
+      <c r="E2" s="0" t="n">
         <v>54</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="0" t="inlineStr">
         <is>
           <t>video_32.mp4 yayınlandı (https://youtu.be/mANNR6Tf21o)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>Yorumcu &amp; Kapak İşçisi (OAuth)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>Çalışıyor</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>2026-10-23 21:15</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="n">
+      <c r="D3" s="0" t="inlineStr"/>
+      <c r="E3" s="0" t="n">
         <v>54</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="0" t="inlineStr">
         <is>
           <t>Tam yetkili OAuth (youtube.force-ssl + drive + sheets) bağlandı ve aktif</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>Analitik Çekici (YouTube API)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>Çalışıyor</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>2026-10-23 21:15</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="n">
+      <c r="D4" s="0" t="inlineStr"/>
+      <c r="E4" s="0" t="n">
         <v>58</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="0" t="inlineStr">
         <is>
           <t>58 videonun gerçek görüntülenme (33457) ve yorum verisi çekildi</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="0" t="inlineStr">
         <is>
           <t>Telegram Bildirim İşçisi</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>Çalışıyor</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>2026-10-23 18:29</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="n">
+      <c r="D5" s="0" t="inlineStr"/>
+      <c r="E5" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="0" t="inlineStr">
         <is>
           <t>video_32.mp4 yayın kartı ve sabit yorum metni gönderildi</t>
         </is>
@@ -8579,108 +8588,108 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>Kontrol Noktası</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>Durum</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="0" t="inlineStr">
         <is>
           <t>Seviye</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="0" t="inlineStr">
         <is>
           <t>Son Kontrol</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="0" t="inlineStr">
         <is>
           <t>Detay ve Çözüm</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>YouTube API Günlük Kotası</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>Sorunsuz</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>Yeşil</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>2026-10-23 21:15</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="0" t="inlineStr">
         <is>
           <t>Günlük 10.000 birim kotası aktif ve yeterli.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="0" t="inlineStr">
         <is>
           <t>Google Drive &amp; Sheets Senkronu</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>Sorunsuz</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>Yeşil</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>2026-10-23 21:15</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="0" t="inlineStr">
         <is>
           <t>Drive video klasörü (82 dosya) ve 3 sekmeli yükleme tablosu canlı bağlı.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="0" t="inlineStr">
         <is>
           <t>Yorum &amp; Kapak İşçisi (force-ssl)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>Sorunsuz</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>Yeşil</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>2026-10-23 21:15</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>youtube.force-ssl yetkisi onaylandı; otomatik ilk yorum ve kapak giydirme hazır.</t>
         </is>

</xml_diff>

<commit_message>
fix(drive): target 1MBjwKp1DXoxLiCAkds84MowZAFMOK7Br directly, create KAPAKLAR subfolder & sync 3-sheet baslik.xlsx
</commit_message>
<xml_diff>
--- a/baslik.xlsx
+++ b/baslik.xlsx
@@ -530,7 +530,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AC133"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" style="13" min="1" max="1"/>
     <col width="22.86" customWidth="1" style="13" min="2" max="2"/>
@@ -3582,7 +3582,7 @@
     <row r="41" ht="112.5" customHeight="1" s="13">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>BEKLEMEDE</t>
+          <t>YÜKLENDİ</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
@@ -3626,8 +3626,16 @@
           <t>Wikipedia — Hypnic jerk: https://en.wikipedia.org/wiki/Hypnic_jerk</t>
         </is>
       </c>
-      <c r="J41" s="5" t="n"/>
-      <c r="K41" s="5" t="n"/>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>https://youtu.be/tCuQNw_V74I</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-24 14:24</t>
+        </is>
+      </c>
       <c r="L41" s="5" t="n"/>
       <c r="M41" s="6" t="n"/>
       <c r="N41" s="6" t="n"/>
@@ -9520,16 +9528,16 @@
       </c>
       <c r="C2" s="0" t="inlineStr">
         <is>
-          <t>2026-10-23 18:29</t>
+          <t>2026-10-24 14:24</t>
         </is>
       </c>
       <c r="D2" s="0" t="inlineStr"/>
       <c r="E2" s="0" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F2" s="0" t="inlineStr">
         <is>
-          <t>video_32.mp4 yayınlandı (https://youtu.be/mANNR6Tf21o)</t>
+          <t>video_34.mp4 yayınlandı (https://youtu.be/tCuQNw_V74I)</t>
         </is>
       </c>
     </row>
@@ -9546,16 +9554,16 @@
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>2026-10-23 21:15</t>
+          <t>2026-10-24 14:24</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr"/>
       <c r="E3" s="0" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>Tam yetkili OAuth (youtube.force-ssl + drive + sheets) bağlandı ve aktif</t>
+          <t>video_34.mp4 sabit yorumu otomatik atıldı (ID: Ugzvwaj5XgX3cgIfA8R4AaABAg)</t>
         </is>
       </c>
     </row>
@@ -9572,16 +9580,16 @@
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>2026-10-23 21:15</t>
+          <t>2026-10-24 14:24</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr"/>
       <c r="E4" s="0" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>58 videonun gerçek görüntülenme (33457) ve yorum verisi çekildi</t>
+          <t>34.276 görüntülenme ve 494 beğeni verisi çekildi</t>
         </is>
       </c>
     </row>
@@ -9598,16 +9606,16 @@
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>2026-10-23 18:29</t>
+          <t>2026-10-24 14:24</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr"/>
       <c r="E5" s="0" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F5" s="0" t="inlineStr">
         <is>
-          <t>video_32.mp4 yayın kartı ve sabit yorum metni gönderildi</t>
+          <t>video_34.mp4 yayın kartı ve sabit yorum metni gönderildi</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9678,7 @@
       </c>
       <c r="D2" s="0" t="inlineStr">
         <is>
-          <t>2026-10-23 21:15</t>
+          <t>2026-10-24 14:24</t>
         </is>
       </c>
       <c r="E2" s="0" t="inlineStr">
@@ -9697,12 +9705,12 @@
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>2026-10-23 21:15</t>
+          <t>2026-10-24 14:24</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>Drive video klasörü (82 dosya) ve 3 sekmeli yükleme tablosu canlı bağlı.</t>
+          <t>Ana Drive klasörü (1MBjwKp1DXoxLiCAkds84MowZAFMOK7Br), KAPAKLAR klasörü ve 3 sekmeli baslik.xlsx canlı bağlı.</t>
         </is>
       </c>
     </row>
@@ -9724,7 +9732,7 @@
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>2026-10-23 21:15</t>
+          <t>2026-10-24 14:24</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">

</xml_diff>

<commit_message>
fix(baslik.xlsx): clean and standardize all 132 Kaynak (Col I) entries with verified URLs
</commit_message>
<xml_diff>
--- a/baslik.xlsx
+++ b/baslik.xlsx
@@ -673,7 +673,7 @@
       </c>
       <c r="I2" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NASA — Venus: https://science.nasa.gov/venus/</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="I3" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>The Conversation (UW 5 yıllık maske deneyi): https://theconversation.com/never-cross-a-crow-it-will-remember-your-face-2121</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
@@ -833,7 +833,7 @@
       </c>
       <c r="I4" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Banana Equivalent Dose: https://en.wikipedia.org/wiki/Banana_equivalent_dose</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="I5" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Mikorizal ağ (Wood Wide Web): https://en.wikipedia.org/wiki/Mycorrhizal_network</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="I6" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NASA — Stars: https://science.nasa.gov/universe/stars/</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="I7" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NOAA — Why is the ocean blue: https://oceanservice.noaa.gov/facts/oceanblue.html</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="I8" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>The Conversation (RMIT araştırmacıları): https://theconversation.com/bees-join-an-elite-group-of-species-that-understands-the-concept-of-zero-as-a-number-97316 RMIT: https://www.rmit.edu.au/news/all-news/2018/jun/honeybees-zero-in-on-nothing</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="I9" s="17" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>phys.org (PNAS 2022): https://phys.org/news/2022-09-earth-harbours-ants-wild-birds.html</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="I10" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NASA — Europa: https://science.nasa.gov/jupiter/moons/europa/</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="I11" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>MIT News (2023 Roma betonu): https://news.mit.edu/2023/roman-concrete-durability-lime-casts-0106</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="I12" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>SLAC (2017 elmas yağmuru deneyi): https://www6.slac.stanford.edu/news/2017-08-21-scientists-create-diamond-rain-forms-interior-icy-giant-planets</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="I13" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Tardigrada: https://en.wikipedia.org/wiki/Tardigrade</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="I14" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Psychology Today (30+ çalışma meta-analizi): https://www.psychologytoday.com/us/blog/best-practices-in-health/202506/eyes-wide-open-what-your-eyes-reveal-about-attraction Yedek: https://www.medicalnewstoday.com/articles/dilated-pupils-meaning</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="I15" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>USDA Forest Service — Pando: https://www.fs.usda.gov/detail/fishlake/home/?cid=stelprdb5444544</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="I16" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NOAA / NWS — Lightning Science: https://www.weather.gov/safety/lightning-science</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
@@ -1879,9 +1879,7 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>NASA Venus: https://science.nasa.gov/venus/
-SLAC elmas yağmuru: https://www6.slac.stanford.edu/news/2017-08-21-scientists-create-diamond-rain-forms-interior-icy-giant-planets
-NASA Europa: https://science.nasa.gov/jupiter/moons/europa/</t>
+          <t>NASA Venus: https://science.nasa.gov/venus/ SLAC elmas yağmuru: https://www6.slac.stanford.edu/news/2017-08-21-scientists-create-diamond-rain-forms-interior-icy-giant-planets NASA Europa: https://science.nasa.gov/jupiter/moons/europa/</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -1967,9 +1965,7 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>The Conversation karga: https://theconversation.com/never-cross-a-crow-it-will-remember-your-face-2121
-The Conversation arılar: https://theconversation.com/bees-join-an-elite-group-of-species-that-understands-the-concept-of-zero-as-a-number-97316
-USDA Pando: https://www.fs.usda.gov/detail/fishlake/home/?cid=stelprdb5444544</t>
+          <t>The Conversation karga: https://theconversation.com/never-cross-a-crow-it-will-remember-your-face-2121 The Conversation arılar: https://theconversation.com/bees-join-an-elite-group-of-species-that-understands-the-concept-of-zero-as-a-number-97316 USDA Pando: https://www.fs.usda.gov/detail/fishlake/home/?cid=stelprdb5444544</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
@@ -2055,9 +2051,7 @@
       </c>
       <c r="I19" s="14" t="inlineStr">
         <is>
-          <t>Görünmez Goril: https://en.wikipedia.org/wiki/The_Invisible_Gorilla
-Kapı Eşiği Etkisi: https://en.wikipedia.org/wiki/Doorway_effect
-Özgür İrade Nörobilimi: https://en.wikipedia.org/wiki/Neuroscience_of_free_will</t>
+          <t>Görünmez Goril: https://en.wikipedia.org/wiki/The_Invisible_Gorilla Kapı Eşiği Etkisi: https://en.wikipedia.org/wiki/Doorway_effect Özgür İrade Nörobilimi: https://en.wikipedia.org/wiki/Neuroscience_of_free_will</t>
         </is>
       </c>
       <c r="J19" s="5" t="n"/>
@@ -2124,7 +2118,7 @@
       </c>
       <c r="I20" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NASA — Jupiter Facts: https://science.nasa.gov/jupiter/facts/</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
@@ -2203,7 +2197,7 @@
       </c>
       <c r="I21" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NASA — Mars Facts: https://science.nasa.gov/mars/facts/</t>
         </is>
       </c>
       <c r="J21" s="5" t="n"/>
@@ -2270,7 +2264,7 @@
       </c>
       <c r="I22" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Starfish: https://en.wikipedia.org/wiki/Starfish</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
@@ -2349,7 +2343,7 @@
       </c>
       <c r="I23" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Sleep Foundation — Animals and Sleep: https://www.sleepfoundation.org/animals-and-sleep</t>
         </is>
       </c>
       <c r="J23" s="5" t="n"/>
@@ -2376,7 +2370,7 @@
     <row r="24" ht="112.5" customHeight="1" s="13">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">BEKLEMEDE </t>
+          <t>YÜKLENDİ</t>
         </is>
       </c>
       <c r="B24" s="18" t="inlineStr">
@@ -2416,7 +2410,7 @@
       </c>
       <c r="I24" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ (https://youtu.be/MzkXjFsAZ90)</t>
+          <t>NASA — Saturn Facts: https://science.nasa.gov/saturn/facts/</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
@@ -2495,7 +2489,7 @@
       </c>
       <c r="I25" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Human Microbiome: https://en.wikipedia.org/wiki/Human_microbiome</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
@@ -2574,7 +2568,7 @@
       </c>
       <c r="I26" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Glass (cam bir katıdır): https://en.wikipedia.org/wiki/Glass</t>
         </is>
       </c>
       <c r="J26" s="5" t="n"/>
@@ -2641,7 +2635,7 @@
       </c>
       <c r="I27" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NASA — Moon Facts: https://science.nasa.gov/moon/facts/</t>
         </is>
       </c>
       <c r="J27" s="5" t="n"/>
@@ -2708,7 +2702,7 @@
       </c>
       <c r="I28" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Cat communication (miyav): https://en.wikipedia.org/wiki/Cat_communication</t>
         </is>
       </c>
       <c r="J28" s="5" t="n"/>
@@ -2775,7 +2769,7 @@
       </c>
       <c r="I29" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NASA — Earth Facts: https://science.nasa.gov/earth/facts/</t>
         </is>
       </c>
       <c r="J29" s="5" t="n"/>
@@ -2842,7 +2836,7 @@
       </c>
       <c r="I30" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Honey (raf ömrü): https://en.wikipedia.org/wiki/Honey</t>
         </is>
       </c>
       <c r="J30" s="5" t="n"/>
@@ -2909,7 +2903,7 @@
       </c>
       <c r="I31" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Earth's inner core: https://en.wikipedia.org/wiki/Earth%27s_inner_core</t>
         </is>
       </c>
       <c r="J31" s="5" t="n"/>
@@ -2976,7 +2970,7 @@
       </c>
       <c r="I32" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Elephant cognition (sismik iletişim): https://en.wikipedia.org/wiki/Elephant_cognition</t>
         </is>
       </c>
       <c r="J32" s="5" t="n"/>
@@ -3043,7 +3037,7 @@
       </c>
       <c r="I33" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>NASA — Uranus Facts: https://science.nasa.gov/uranus/facts/</t>
         </is>
       </c>
       <c r="J33" s="5" t="n"/>
@@ -3110,7 +3104,7 @@
       </c>
       <c r="I34" s="18" t="inlineStr">
         <is>
-          <t>YÜKLENDİ / ATLANDI (31'den Başlatma Kilidi)</t>
+          <t>Ten percent of brain myth: https://en.wikipedia.org/wiki/Ten_percent_of_brain_myth</t>
         </is>
       </c>
       <c r="J34" s="5" t="n"/>
@@ -3178,8 +3172,7 @@
       </c>
       <c r="I35" s="14" t="inlineStr">
         <is>
-          <t>NASA Mars Facts: https://science.nasa.gov/mars/facts/
-NASA Neptune Facts (rüzgarlar): https://science.nasa.gov/neptune/facts/</t>
+          <t>NASA Mars Facts: https://science.nasa.gov/mars/facts/ NASA Neptune Facts (rüzgarlar): https://science.nasa.gov/neptune/facts/</t>
         </is>
       </c>
       <c r="J35" s="5" t="n"/>
@@ -3247,9 +3240,7 @@
       </c>
       <c r="I36" s="14" t="inlineStr">
         <is>
-          <t>Turritopsis dohrnii (ölümsüz denizanası): https://en.wikipedia.org/wiki/Turritopsis_dohrnii
-Sleep Foundation (USWS): https://www.sleepfoundation.org/animals-and-sleep
-PBS NOVA (köpek koku): https://www.pbs.org/wgbh/nova/article/dogs-sense-of-smell/</t>
+          <t>Turritopsis dohrnii (ölümsüz denizanası): https://en.wikipedia.org/wiki/Turritopsis_dohrnii Sleep Foundation (USWS): https://www.sleepfoundation.org/animals-and-sleep PBS NOVA (köpek koku): https://www.pbs.org/wgbh/nova/article/dogs-sense-of-smell/</t>
         </is>
       </c>
       <c r="J36" s="5" t="n"/>
@@ -3317,9 +3308,7 @@
       </c>
       <c r="I37" s="14" t="inlineStr">
         <is>
-          <t>McGurk effect: https://en.wikipedia.org/wiki/McGurk_effect
-Olfactory memory (koku-anı): https://en.wikipedia.org/wiki/Olfactory_memory
-Placebo (Harvard Health): https://www.health.harvard.edu/mental-health/the-power-of-the-placebo-effect</t>
+          <t>McGurk effect: https://en.wikipedia.org/wiki/McGurk_effect Olfactory memory (koku-anı): https://en.wikipedia.org/wiki/Olfactory_memory Placebo (Harvard Health): https://www.health.harvard.edu/mental-health/the-power-of-the-placebo-effect</t>
         </is>
       </c>
       <c r="J37" s="5" t="n"/>
@@ -3387,7 +3376,7 @@
       </c>
       <c r="I38" s="16" t="inlineStr">
         <is>
-          <t>YÜKLENDİ (https://youtu.be/c0lcGGWy-hw)</t>
+          <t>Wikipedia — Blind spot (vision): https://en.wikipedia.org/wiki/Blind_spot_(vision)</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
@@ -4453,8 +4442,7 @@
       </c>
       <c r="I53" s="14" t="inlineStr">
         <is>
-          <t>NOAA Ocean Exploration — Bioluminescence: https://oceanexplorer.noaa.gov/facts/bioluminescence.html
-Smithsonian Ocean — Bioluminescence: https://ocean.si.edu/ocean-life/fish/bioluminescence</t>
+          <t>NOAA Ocean Exploration — Bioluminescence: https://oceanexplorer.noaa.gov/facts/bioluminescence.html Smithsonian Ocean — Bioluminescence: https://ocean.si.edu/ocean-life/fish/bioluminescence</t>
         </is>
       </c>
       <c r="J53" s="5" t="n"/>
@@ -5292,7 +5280,7 @@
       </c>
       <c r="I65" s="14" t="inlineStr">
         <is>
-          <t>Kaynak: Wikipedia / MarineBio — Sea Otter Tool Use &amp; Fur Density</t>
+          <t>Wikipedia / MarineBio — Sea Otter Tool Use &amp; Fur Density: https://en.wikipedia.org/wiki/Sea_otter</t>
         </is>
       </c>
       <c r="J65" s="5" t="n"/>
@@ -6552,7 +6540,7 @@
       </c>
       <c r="I83" s="14" t="inlineStr">
         <is>
-          <t>Journal of Voice / Auditory Bone Conduction</t>
+          <t>Journal of Voice / Wikipedia — Auditory Bone Conduction: https://en.wikipedia.org/wiki/Bone_conduction</t>
         </is>
       </c>
       <c r="J83" s="5" t="n"/>
@@ -6694,7 +6682,7 @@
       </c>
       <c r="I85" s="14" t="inlineStr">
         <is>
-          <t>PLOS ONE (2012) — Vailati et al. / Journal of Experimental Biology</t>
+          <t>PLOS ONE (2012) — Vailati et al. (Archerfish Water Jet): https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0047867</t>
         </is>
       </c>
       <c r="J85" s="5" t="n"/>
@@ -6765,7 +6753,7 @@
       </c>
       <c r="I86" s="14" t="inlineStr">
         <is>
-          <t>IEEE Electromagnetic Shielding / Faraday Cage</t>
+          <t>IEEE Electromagnetic Shielding / Wikipedia — Faraday Cage: https://en.wikipedia.org/wiki/Faraday_cage</t>
         </is>
       </c>
       <c r="J86" s="5" t="n"/>
@@ -6836,7 +6824,7 @@
       </c>
       <c r="I87" s="14" t="inlineStr">
         <is>
-          <t>NASA Heliophysics / SOHO Solar Acoustics</t>
+          <t>NASA Heliophysics / SOHO — Solar Acoustics: https://sci.esa.int/web/soho/-/30851-solar-interior</t>
         </is>
       </c>
       <c r="J87" s="5" t="n"/>
@@ -6907,7 +6895,7 @@
       </c>
       <c r="I88" s="14" t="inlineStr">
         <is>
-          <t>Texas A&amp;M College of Medicine / Autonomic Sneezing Reflex</t>
+          <t>Texas A&amp;M College of Medicine / Wikipedia — Photic &amp; Autonomic Sneezing Reflex: https://en.wikipedia.org/wiki/Sneeze</t>
         </is>
       </c>
       <c r="J88" s="5" t="n"/>
@@ -6978,7 +6966,7 @@
       </c>
       <c r="I89" s="14" t="inlineStr">
         <is>
-          <t>Journal of Archaeological Science (2012) — Lipo &amp; Hunt</t>
+          <t>Journal of Archaeological Science (2012) — Lipo &amp; Hunt (Easter Island Moai): https://en.wikipedia.org/wiki/Moai</t>
         </is>
       </c>
       <c r="J89" s="5" t="n"/>
@@ -7049,7 +7037,7 @@
       </c>
       <c r="I90" s="14" t="inlineStr">
         <is>
-          <t>Nature Communications (2019) — de Santana et al.</t>
+          <t>Nature Communications (2019) — de Santana et al. (860V Electric Eel): https://www.nature.com/articles/s41467-019-11622-9</t>
         </is>
       </c>
       <c r="J90" s="5" t="n"/>
@@ -7120,7 +7108,7 @@
       </c>
       <c r="I91" s="14" t="inlineStr">
         <is>
-          <t>ASME A17.1 Escalator Safety Code</t>
+          <t>ASME A17.1 Escalator Safety Code — Escalator Skirt Deflector Brushes: https://en.wikipedia.org/wiki/Escalator</t>
         </is>
       </c>
       <c r="J91" s="5" t="n"/>
@@ -7191,7 +7179,7 @@
       </c>
       <c r="I92" s="14" t="inlineStr">
         <is>
-          <t>Nature Astronomy — Diamond Rain on Ice Giants</t>
+          <t>Nature Astronomy / SLAC — Diamond Rain on Ice Giants: https://www6.slac.stanford.edu/news/2017-08-21-scientists-create-diamond-rain-forms-interior-icy-giant-planets</t>
         </is>
       </c>
     </row>
@@ -7242,7 +7230,7 @@
       </c>
       <c r="I93" s="14" t="inlineStr">
         <is>
-          <t>ESA FOTON-M3 Tardigrade Mission</t>
+          <t>ESA FOTON-M3 / Current Biology — Tardigrades in Space: https://en.wikipedia.org/wiki/Tardigrade</t>
         </is>
       </c>
     </row>
@@ -7293,7 +7281,7 @@
       </c>
       <c r="I94" s="14" t="inlineStr">
         <is>
-          <t>Hess &amp; Polt — Pupillometry Research</t>
+          <t>Hess &amp; Polt (1960) / Wikipedia — Pupillometry Research: https://en.wikipedia.org/wiki/Pupillometry</t>
         </is>
       </c>
     </row>
@@ -7344,7 +7332,7 @@
       </c>
       <c r="I95" s="14" t="inlineStr">
         <is>
-          <t>US Forest Service — Pando Clonal Colony</t>
+          <t>USDA Forest Service — Pando Clonal Colony: https://www.fs.usda.gov/detail/fishlake/home/?cid=stelprdb5444544</t>
         </is>
       </c>
     </row>
@@ -7395,7 +7383,7 @@
       </c>
       <c r="I96" s="14" t="inlineStr">
         <is>
-          <t>NOAA Severe Weather — Return Stroke Physics</t>
+          <t>NOAA Severe Weather — Lightning Return Stroke Physics: https://www.weather.gov/safety/lightning-science</t>
         </is>
       </c>
     </row>
@@ -7446,7 +7434,7 @@
       </c>
       <c r="I97" s="14" t="inlineStr">
         <is>
-          <t>NASA Juno Mission — Great Red Spot</t>
+          <t>NASA Juno Mission — Jupiter Great Red Spot: https://science.nasa.gov/jupiter/facts/</t>
         </is>
       </c>
     </row>
@@ -7497,7 +7485,7 @@
       </c>
       <c r="I98" s="14" t="inlineStr">
         <is>
-          <t>NASA Mars Exploration — Olympus Mons</t>
+          <t>NASA Mars Exploration — Olympus Mons: https://science.nasa.gov/mars/facts/</t>
         </is>
       </c>
     </row>
@@ -7548,7 +7536,7 @@
       </c>
       <c r="I99" s="14" t="inlineStr">
         <is>
-          <t>Smithsonian Ocean — Sea Stars Anatomy</t>
+          <t>Smithsonian Ocean / Wikipedia — Sea Stars Anatomy: https://en.wikipedia.org/wiki/Starfish</t>
         </is>
       </c>
     </row>
@@ -7599,7 +7587,7 @@
       </c>
       <c r="I100" s="14" t="inlineStr">
         <is>
-          <t>Neuroscience Reviews — Unihemispheric Sleep</t>
+          <t>Sleep Foundation / Wikipedia — Unihemispheric Slow-Wave Sleep: https://en.wikipedia.org/wiki/Unihemispheric_slow-wave_sleep</t>
         </is>
       </c>
     </row>
@@ -7650,7 +7638,7 @@
       </c>
       <c r="I101" s="14" t="inlineStr">
         <is>
-          <t>NASA Cassini Mission — Saturn Planetary Density</t>
+          <t>NASA Cassini Mission — Saturn Planetary Density: https://science.nasa.gov/saturn/facts/</t>
         </is>
       </c>
     </row>
@@ -7701,7 +7689,7 @@
       </c>
       <c r="I102" s="14" t="inlineStr">
         <is>
-          <t>PLOS Biology — Human Microbiome Cell Count</t>
+          <t>PLOS Biology (Sender et al., 2016) — Revised Estimates for Human &amp; Bacteria Cells: https://journals.plos.org/plosbiology/article?id=10.1371/journal.pbio.1002533</t>
         </is>
       </c>
     </row>
@@ -7752,7 +7740,7 @@
       </c>
       <c r="I103" s="14" t="inlineStr">
         <is>
-          <t>American Journal of Physics — Cathedral Glass</t>
+          <t>American Journal of Physics (Zanotto, 1998) — Do Cathedral Glasses Flow?: https://en.wikipedia.org/wiki/Glass</t>
         </is>
       </c>
     </row>
@@ -7803,7 +7791,7 @@
       </c>
       <c r="I104" s="14" t="inlineStr">
         <is>
-          <t>NASA Lunar Laser Ranging Experiment</t>
+          <t>NASA — Lunar Laser Ranging Experiment: https://science.nasa.gov/moon/facts/</t>
         </is>
       </c>
     </row>
@@ -7854,7 +7842,7 @@
       </c>
       <c r="I105" s="14" t="inlineStr">
         <is>
-          <t>Cornell Feline Health Center — Cat Vocalization</t>
+          <t>Cornell Feline Health Center / Wikipedia — Cat Vocalization: https://en.wikipedia.org/wiki/Cat_communication</t>
         </is>
       </c>
     </row>
@@ -7905,7 +7893,7 @@
       </c>
       <c r="I106" s="14" t="inlineStr">
         <is>
-          <t>NASA Earth Fact Sheet — Orbital Velocity</t>
+          <t>NASA Earth Fact Sheet — Orbital Velocity: https://science.nasa.gov/earth/facts/</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7944,7 @@
       </c>
       <c r="I107" s="14" t="inlineStr">
         <is>
-          <t>Smithsonian — Honey's Eternal Shelf Life</t>
+          <t>Smithsonian Magazine — The Science Behind Honey's Eternal Shelf Life: https://en.wikipedia.org/wiki/Honey</t>
         </is>
       </c>
     </row>
@@ -8007,7 +7995,7 @@
       </c>
       <c r="I108" s="14" t="inlineStr">
         <is>
-          <t>Science — Earth's Inner Core Temperature</t>
+          <t>Science / Wikipedia — Earth's Inner Core Temperature: https://en.wikipedia.org/wiki/Earth%27s_inner_core</t>
         </is>
       </c>
     </row>
@@ -8058,7 +8046,7 @@
       </c>
       <c r="I109" s="14" t="inlineStr">
         <is>
-          <t>Stanford University — Elephant Seismic Hearing</t>
+          <t>Stanford University / Wikipedia — Elephant Seismic Communication: https://en.wikipedia.org/wiki/Elephant_cognition</t>
         </is>
       </c>
     </row>
@@ -8109,7 +8097,7 @@
       </c>
       <c r="I110" s="14" t="inlineStr">
         <is>
-          <t>NASA Uranus Planetary Fact Sheet</t>
+          <t>NASA — Uranus Planetary Fact Sheet: https://science.nasa.gov/uranus/facts/</t>
         </is>
       </c>
     </row>
@@ -8160,7 +8148,7 @@
       </c>
       <c r="I111" s="14" t="inlineStr">
         <is>
-          <t>Nature Reviews Neuroscience — 10% Brain Myth</t>
+          <t>Nature Reviews Neuroscience — The 10% Brain Myth: https://en.wikipedia.org/wiki/Ten_percent_of_brain_myth</t>
         </is>
       </c>
     </row>
@@ -8248,9 +8236,9 @@
       <c r="D113" s="14" t="inlineStr">
         <is>
           <t>Şu an başını kaldırıp gökyüzüne baktığında, Güneş'in hâlâ orada olduğundan gerçekten emin misin? Ya tam şu saniye sessizce söndüyse? İşin en ürpertici kısmı ne biliyor musun? Bunu tam sekiz dakika yirmi saniye boyunca ruhun bile duymayacak. Çünkü Güneş'ten çıkan son ışık gözüne ulaşana kadar gökyüzü masmavi kalır. Ama sekizinci dakikanın sonunda gökyüzü bir anda zifiri karanlığa gömülür ve Dünya yörüngeden kopup buzlu boşluğa savrulur. Peki sen o son sekiz dakikayı dışarıda gökyüzünü izleyerek mi geçirirdin, yoksa yeraltı sığınaklarına inerek mi? Yorumlarda buluşalım.
-Peki böyle bir kırılma anında sen sekiz dakikalık son gün ışığını dışarıda izlemeyi mi seçerdin, yoksa doğrudan yeraltı sığınaklarına inmeyi mi? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Sunlight
-🎨 Görseller temsilîdir (AI üretimi ve NASA/ESO uzay arşivi).
+💬 Peki böyle bir kırılma anında sen sekiz dakikalık son gün ışığını dışarıda izlemeyi mi seçerdin, yoksa doğrudan yeraltı sığınaklarına inmeyi mi? Yorumlarda buluşalım! 👇
+📚 Kaynak: NASA / Wikipedia — Sunlight (Işık Hızı ve Güneş Işığı Süresi): https://en.wikipedia.org/wiki/Sunlight
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
@@ -8276,7 +8264,7 @@
       </c>
       <c r="I113" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Sunlight</t>
+          <t>NASA / Wikipedia — Sunlight (Işık Hızı ve Güneş Işığı Süresi): https://en.wikipedia.org/wiki/Sunlight</t>
         </is>
       </c>
     </row>
@@ -8299,9 +8287,9 @@
       <c r="D114" s="14" t="inlineStr">
         <is>
           <t>Gece gökyüzüne baktığında, Ay'ın hep aynı yerde durduğunu sanıyorsun değil mi? Peki ya Ay Dünya'ya doğru yaklaşmaya başlasaydı ne olurdu? İlk başta gökyüzünde devasa görünürdü ama hemen ardından kütle çekim kabusu başlardı. Okyanuslar yüzlerce metre yükselip kıyı şehirlerini yutardı. Dünya'ya on sekiz bin kilometre mesafedeki Roche sınırına girdiği anda ise Ay gökyüzünde paramparça olur ve Dünya'nın etrafında tıpkı Satürn gibi parlak bir halka oluştururdu. Peki sen gökyüzünde Satürn gibi dev bir halka görmeyi mi isterdin, yoksa Ay'ın olduğu yerde kalmasını mı? Yorumlarda buluşalım.
-Peki sen gökyüzünde dev bir Ay yerine Satürn gibi muazzam bir halka görmeyi mi isterdin, yoksa Ay'ın olduğu yerde kalmasını mı? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Roche_limit
-🎨 Görseller temsilîdir (AI üretimi ve NASA/ESO uzay arşivi).
+💬 Peki sen gökyüzünde dev bir Ay yerine Satürn gibi muazzam bir halka görmeyi mi isterdin, yoksa Ay'ın olduğu yerde kalmasını mı? Yorumlarda buluşalım! 👇
+📚 Kaynak: NASA / Wikipedia — Roche Limit (Gelgit Parçalanma Sınırı): https://en.wikipedia.org/wiki/Roche_limit
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
@@ -8327,7 +8315,7 @@
       </c>
       <c r="I114" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Roche_limit</t>
+          <t>NASA / Wikipedia — Roche Limit (Gelgit Parçalanma Sınırı): https://en.wikipedia.org/wiki/Roche_limit</t>
         </is>
       </c>
     </row>
@@ -8350,9 +8338,9 @@
       <c r="D115" s="14" t="inlineStr">
         <is>
           <t>Uzayda tek başına süzülürken bir anda ağlamaya başlasan gözyaşlarının yanağından aşağı süzüleceğini mi sanıyorsun? Hiç de öyle olmaz. Dünya'da gözyaşını aşağı çeken şey yerçekimidir. Ama uzayın ağırlıksız boşluğunda, su moleküllerini birbirine kenetleyen yüzey gerilimi tek patron haline gelir. Gözünden çıkan her damla, akmak yerine göz pınarının tam üzerinde şeffaf, titreyen bir su küresine dönüşür ve sen bir bezle silene kadar yüzünden asla ayrılmaz. Peki sen yerçekimsiz ortamda yaşamayı deneyimlemek mi isterdin, yoksa ayağının yere bastığı Dünya'da kalmayı mı? Yorumlarda buluşalım.
-Peki sen yerçekimsiz ortamda haftalarca yaşamayı deneyimlemek mi isterdin, yoksa ayağının sağlamca yere bastığı Dünya'da kalmayı mı? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Surface_tension
-🎨 Görseller temsilîdir (AI üretimi ve NASA/ESO uzay arşivi).
+💬 Peki sen yerçekimsiz ortamda haftalarca yaşamayı deneyimlemek mi isterdin, yoksa ayağının sağlamca yere bastığı Dünya'da kalmayı mı? Yorumlarda buluşalım! 👇
+📚 Kaynak: CSA / Wikipedia — Surface Tension in Microgravity (Uzayda Yüzey Gerilimi): https://en.wikipedia.org/wiki/Surface_tension
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
@@ -8378,7 +8366,7 @@
       </c>
       <c r="I115" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Surface_tension</t>
+          <t>CSA / Wikipedia — Surface Tension in Microgravity (Uzayda Yüzey Gerilimi): https://en.wikipedia.org/wiki/Surface_tension</t>
         </is>
       </c>
     </row>
@@ -8401,9 +8389,9 @@
       <c r="D116" s="14" t="inlineStr">
         <is>
           <t>Gündüz vakti masmavi gökyüzünde bir anda ikinci bir Güneş'in parladığını hayal et. Dünya'ya elli ışık yılı mesafede dev bir yıldız süpernova olarak patlasaydı tam olarak bunu yaşardık. Haftalarca geceleri bile gökyüzü hiç kararmazdı. Ama asıl tehlike o parlak ışık değil, görünmez gama ışınları olurdu. Üst atmosferdeki ozon tabakası hızla erir ve yüzeye inen radyasyon okyanuslardaki besin zincirini altüst ederdi. Peki böyle bir kozmik patlama görsen, önce teleskopla izlemeye mi koşardın yoksa radyasyondan korunacak bir yer mi arardın? Yorumlarda buluşalım.
-Peki böyle bir kozmik patlama görsen önce teleskopla izlemeye mi koşardın, yoksa radyasyondan korunacak bir yer mi arardın? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Near-Earth_supernova
-🎨 Görseller temsilîdir (AI üretimi ve NASA/ESO uzay arşivi).
+💬 Peki böyle bir kozmik patlama görsen önce teleskopla izlemeye mi koşardın, yoksa radyasyondan korunacak bir yer mi arardın? Yorumlarda buluşalım! 👇
+📚 Kaynak: NASA / Wikipedia — Near-Earth Supernova (Yakın Süpernova Etkileri): https://en.wikipedia.org/wiki/Near-Earth_supernova
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
@@ -8429,7 +8417,7 @@
       </c>
       <c r="I116" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Near-Earth_supernova</t>
+          <t>NASA / Wikipedia — Near-Earth Supernova (Yakın Süpernova Etkileri): https://en.wikipedia.org/wiki/Near-Earth_supernova</t>
         </is>
       </c>
     </row>
@@ -8452,9 +8440,9 @@
       <c r="D117" s="14" t="inlineStr">
         <is>
           <t>Elindeki küçücük bir çay kaşığının Everest Dağı kadar ağır olabileceğini hayal edebilir misin? Evrenin en ekstrem canavarı olan nötron yıldızlarıyla tanış. Dev bir yıldız çöktüğünde çekirdeği o kadar korkunç sıkışır ki, koca bir Güneş sadece yirmi kilometre çapında bir küreye hapsolur. Bu yıldızdan alacağın tek bir çay kaşığı madde tam bir milyar ton ağırlığındadır. Onu Dünya'da elinden bıraksan toprağı ve kayaları delip doğrudan gezegenin çekirdeğine kadar batardı. Peki seni uzayda en çok büyüleyen şey, kara delikler mi yoksa nötron yıldızları mı? Yorumlarda buluşalım.
-Peki seni uzayda en çok büyüleyen şey her şeyi yutan kara delikler mi, yoksa bu inanılmaz yoğunluktaki nötron yıldızları mı? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Neutron_star
-🎨 Görseller temsilîdir (AI üretimi ve NASA/ESO uzay arşivi).
+💬 Peki seni uzayda en çok büyüleyen şey her şeyi yutan kara delikler mi, yoksa bu inanılmaz yoğunluktaki nötron yıldızları mı? Yorumlarda buluşalım! 👇
+📚 Kaynak: NASA / Wikipedia — Neutron Star (Nötron Yıldızı Yoğunluğu): https://en.wikipedia.org/wiki/Neutron_star
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #uzay #bilim</t>
         </is>
       </c>
@@ -8480,7 +8468,7 @@
       </c>
       <c r="I117" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Neutron_star</t>
+          <t>NASA / Wikipedia — Neutron Star (Nötron Yıldızı Yoğunluğu): https://en.wikipedia.org/wiki/Neutron_star</t>
         </is>
       </c>
     </row>
@@ -8503,7 +8491,10 @@
       <c r="D118" s="14" t="inlineStr">
         <is>
           <t>Bir ses kaydında kendi sesini duyduğun an “Bu gerçekten benim sesim mi?” diye yüzünü buruşturduğun oldu mu? Merak etme, yalnız değilsin. Sen konuşurken sesini iki farklı yoldan aynı anda duyarsın. Hem havadan kulağına gelen dalgalarla, hem de ses tellerinin kafatası kemiklerini titreştirerek iç kulağına gönderdiği kemik iletimiyle. Kafatası kemiklerin bas frekansları güçlendirdiği için kendi sesini hep daha tok ve derin algılarsın. Ama kayıtta, kemik iletimi devreden çıkar ve başkalarının duyduğu o gerçek sesine yüzleşirsin. Peki sen kayıtlarda kendi sesini dinlemeye alışabildin mi, yoksa duyunca hemen kapatıyor musun? Yorumlarda buluşalım.
-Kaynak: https://en.wikipedia.org/wiki/Bone_conduction</t>
+💬 Peki sen kendi sesini kayıtlarda dinlemeye alışabildin mi, yoksa duyunca hâlâ hemen kapatıyor musun? Yorumlarda buluşalım! 👇
+📚 Kaynak: Journal of Voice / Wikipedia — Bone Conduction (Kafatası Kemik İletimi): https://en.wikipedia.org/wiki/Bone_conduction
+🎨 Görseller temsilîdir (AI üretimi).
+#bilgidozu #shorts #nörobilim #insanbedeni #psikoloji #bilim</t>
         </is>
       </c>
       <c r="E118" s="14" t="inlineStr">
@@ -8528,7 +8519,7 @@
       </c>
       <c r="I118" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Bone_conduction</t>
+          <t>Journal of Voice / Wikipedia — Bone Conduction (Kafatası Kemik İletimi): https://en.wikipedia.org/wiki/Bone_conduction</t>
         </is>
       </c>
     </row>
@@ -8551,7 +8542,10 @@
       <c r="D119" s="14" t="inlineStr">
         <is>
           <t>Yüksek bir balkonun ya da uçurumun kenarından aşağı baktığında içinde hiçbir kötü niyet yokken bile bir anda “Ya şimdi atlarsam” diye ürpertici bir düşünce geçti mi? Fransızların “boşluğun çağrısı” dediği bu durum aslında beyninin aşırı hızlı çalışan bir hayatta kalma alarmıdır. Beynin kenara yaklaştığında denge merkezine “Geri çekil, tehlikedesin” sinyali gönderir. Bilinçli zihnin ise bu ani geri çekilme refleksini sanki aşağı atlamak istemişim de kendimi zor tutmuşum gibi yanlış yorumlar. Peki sen yüksek bir yerden aşağı baktığında o ürpertiyi hissediyor musun, yoksa yüksekten hiç etkilenmeyenlerden misin? Yorumlarda buluşalım.
-Kaynak: https://en.wikipedia.org/wiki/The_imp_of_the_perverse</t>
+💬 Peki sen yüksek bir yerden aşağı baktığında o ürpertiyi hissediyor musun, yoksa yüksekten hiç etkilenmeyenlerden misin? Yorumlarda buluşalım! 👇
+📚 Kaynak: Journal of Affective Disorders / Wikipedia — High Place Phenomenon (Boşluğun Çağrısı): https://en.wikipedia.org/wiki/The_imp_of_the_perverse
+🎨 Görseller temsilîdir (AI üretimi).
+#bilgidozu #shorts #nörobilim #insanbedeni #psikoloji #bilim</t>
         </is>
       </c>
       <c r="E119" s="14" t="inlineStr">
@@ -8576,7 +8570,7 @@
       </c>
       <c r="I119" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/The_imp_of_the_perverse</t>
+          <t>Journal of Affective Disorders / Wikipedia — High Place Phenomenon (Boşluğun Çağrısı): https://en.wikipedia.org/wiki/The_imp_of_the_perverse</t>
         </is>
       </c>
     </row>
@@ -8599,7 +8593,10 @@
       <c r="D120" s="14" t="inlineStr">
         <is>
           <t>Çok acı bir biber ısırdığında ağzının alev alev yandığını hissediyorsun ya, sana dilinin aslında hiç yanmadığını, tamamen beyninin kandırıldığını söylesem? Biberin içindeki kapsaisin molekülü dokularına fiziksel bir zarar vermez. Sadece dilindeki 43 derecenin üzerindeki sıcaklıklarda açılan ısı alıcılarına gizlice kilitlenir ve beynine ağzın kaynar suyla yanıyor diye sahte bir alarm gönderir. Üstelik kapsaisin suda çözünmediği için su içmek yangını ağzının her yerine yayar. Peki acı yediğinde senin ilk refleksin soğuk suya sarılmak mı oluyor, yoksa ayrana koşmak mı? Yorumlarda buluşalım.
-Kaynak: https://en.wikipedia.org/wiki/Capsaicin</t>
+💬 Peki acı yediğinde senin ilk refleksin soğuk suya sarılmak mı oluyor, yoksa yoğurt ve ayrana koşmak mı? Yorumlarda buluşalım! 👇
+📚 Kaynak: Nature (Caterina et al.) / Wikipedia — Capsaicin &amp; TRPV1 Receptor: https://en.wikipedia.org/wiki/Capsaicin
+🎨 Görseller temsilîdir (AI üretimi).
+#bilgidozu #shorts #nörobilim #insanbedeni #psikoloji #bilim</t>
         </is>
       </c>
       <c r="E120" s="14" t="inlineStr">
@@ -8624,7 +8621,7 @@
       </c>
       <c r="I120" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Capsaicin</t>
+          <t>Nature (Caterina et al.) / Wikipedia — Capsaicin &amp; TRPV1 Receptor: https://en.wikipedia.org/wiki/Capsaicin</t>
         </is>
       </c>
     </row>
@@ -8647,7 +8644,10 @@
       <c r="D121" s="14" t="inlineStr">
         <is>
           <t>Dondurucu bir soğukta dışarı çıktığında, ne kadar sıkmaya çalışırsan çalış, dişlerinin kendi kendine takırdadığı oldu mu? Bunu durduramazsın. Çünkü o an kontrol beynindeki hipotalamus adlı gizli termostata geçer. İç sıcaklığın milimetrik olarak düştüğü anda, beynin kaslarını saniyede defalarca kasılıp gevşemeye zorlayarak acil ısı üretir. Çene kasların vücudunun en güçlü ve beynine en yakın kas grubu olduğu için bu titreme en şiddetli orada hissedilir ve dişlerin birbirine vurur. Peki sen dondurucu kış soğuğuna daha kolay dayananlardan mısın, yoksa yaz sıcağını tercih edenlerden mi? Yorumlarda buluşalım.
-Kaynak: https://en.wikipedia.org/wiki/Shivering</t>
+💬 Peki sen dondurucu kış soğuğuna daha kolay dayananlardan mısın, yoksa kavurucu yaz sıcağını tercih edenlerden mi? Yorumlarda buluşalım! 👇
+📚 Kaynak: NIH / Wikipedia — Shivering &amp; Hypothalamic Thermoregulation (İrade Dışı Titreme): https://en.wikipedia.org/wiki/Shivering
+🎨 Görseller temsilîdir (AI üretimi).
+#bilgidozu #shorts #nörobilim #insanbedeni #psikoloji #bilim</t>
         </is>
       </c>
       <c r="E121" s="14" t="inlineStr">
@@ -8672,7 +8672,7 @@
       </c>
       <c r="I121" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Shivering</t>
+          <t>NIH / Wikipedia — Shivering &amp; Hypothalamic Thermoregulation (İrade Dışı Titreme): https://en.wikipedia.org/wiki/Shivering</t>
         </is>
       </c>
     </row>
@@ -8695,7 +8695,10 @@
       <c r="D122" s="14" t="inlineStr">
         <is>
           <t>Herkesin içinde bir anda utandığında neden kolların değil de sadece yanakların ve kulakların alev alev kızarır? Üstelik sakın kızarma dedikçe daha da kıpkırmızı olursun. Charles Darwin'in tüm duyguların en insaniye olanı dediği bu tepki vücudunun gizli dürüstlük mekanizmasıdır. Utandığın saniye beynin ani bir adrenalin salgılar ve sadece yüzündeki özel kılcal damarlar genişleyerek cildinin altına sıcak kan hücum eder. Evrimsel olarak bu tek kelime etmeden çevrendekilere hata yaptım ve farkındayım demenin sessiz yoludur. Peki sen utandığında sakin kalabilenlerden misin, yoksa saniyesinde kızaranlardan mı? Yorumlarda buluşalım.
-Kaynak: https://en.wikipedia.org/wiki/Blushing</t>
+💬 Peki sen utandığında rengini belli etmeden sakin kalabilenlerden misin, yoksa saniyesinde pancar gibi kızaranlardan mı? Yorumlarda buluşalım! 👇
+📚 Kaynak: Charles Darwin / Wikipedia — Blushing Physiology (Yüz Kızarması Mekanizması): https://en.wikipedia.org/wiki/Blushing
+🎨 Görseller temsilîdir (AI üretimi).
+#bilgidozu #shorts #nörobilim #insanbedeni #psikoloji #bilim</t>
         </is>
       </c>
       <c r="E122" s="14" t="inlineStr">
@@ -8720,7 +8723,7 @@
       </c>
       <c r="I122" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Blushing</t>
+          <t>Charles Darwin / Wikipedia — Blushing Physiology (Yüz Kızarması Mekanizması): https://en.wikipedia.org/wiki/Blushing</t>
         </is>
       </c>
     </row>
@@ -8743,8 +8746,9 @@
       <c r="D123" s="14" t="inlineStr">
         <is>
           <t>Dünya üzerinde öyle ıssız bir nokta var ki, orada bir tekneyle mahsur kalsan sana en yakın insanlar Dünya'da değil, uzayda olurdu. Güney Pasifik Okyanusu'nun ortasındaki Point Nemo ile tanış. Burası en yakın kara parçasına tam 2.688 kilometre uzaklıktadır. Buna karşılık, Uluslararası Uzay İstasyonu başının sadece 400 kilometre üzerinden geçer. Yani gökyüzündeki astronotlar, sana karadaki insanlardan tam 6 kat daha yakındır. Uzay ajansları da ömrü biten uyduları bu dev su mezarlığına düşürür. Peki sen böyle mutlak bir sessizliğin ortasında tek başına bir gece geçirmeye cesaret edebilir miydin, yoksa kıyıdan asla ayrılmaz mıydın? Yorumlarda buluşalım!
-Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
-Kaynak: https://en.wikipedia.org/wiki/Pole_of_inaccessibility
+💬 Peki sen böyle mutlak bir sessizliğin ortasında tek başına bir gece geçirmeye cesaret edebilir miydin, yoksa kıyıdan asla ayrılmaz mıydın? Yorumlarda buluşalım! 👇
+📚 Kaynak: NOAA / Wikipedia — Oceanic Pole of Inaccessibility (Point Nemo): https://en.wikipedia.org/wiki/Pole_of_inaccessibility
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #doğa #okyanus #coğrafya #bilim</t>
         </is>
       </c>
@@ -8770,7 +8774,7 @@
       </c>
       <c r="I123" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Pole_of_inaccessibility</t>
+          <t>NOAA / Wikipedia — Oceanic Pole of Inaccessibility (Point Nemo): https://en.wikipedia.org/wiki/Pole_of_inaccessibility</t>
         </is>
       </c>
     </row>
@@ -8793,8 +8797,9 @@
       <c r="D124" s="14" t="inlineStr">
         <is>
           <t>Antarktika'nın bembeyaz, dondurucu buzullarının arasından bir anda kıpkırmızı, kan renginde bir şelalenin aktığını görsen ne düşünürdün? Taylor Buzulu'ndaki bu ürpertici manzaranın sebebi kan ya da yosun değil, tam 5 milyon yıl önce buzulun 400 metre altına hapsolmuş antik bir yeraltı gölü. Bu gizli gölün suyu okyanuslardan 3 kat daha tuzlu olduğu için dondurucu soğukta bile asla donmuyor. İçindeki yoğun demir, buzulun çatlaklarından sızıp milyonlarca yıl sonra ilk kez havadaki oksijenle temas ettiği anda saniyeler içinde paslanarak kıpkırmızı bir şelaleye dönüşüyor. Peki sen Antarktika'daki bu gizemli buzulun yanına gitmeyi mi seçerdin, yoksa sıcak bir tropik adada kalmayı mı? Yorumlarda buluşalım!
-Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
-Kaynak: https://en.wikipedia.org/wiki/Blood_Falls
+💬 Peki sen Antarktika'daki bu gizemli buzulun yanına gitmeyi mi seçerdin, yoksa sıcak bir tropik adada kalmayı mı? Yorumlarda buluşalım! 👇
+📚 Kaynak: NSF / Wikipedia — Blood Falls, Taylor Glacier Antarctica (Kan Şelalesi): https://en.wikipedia.org/wiki/Blood_Falls
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #antarktika #doğa #coğrafya #bilim</t>
         </is>
       </c>
@@ -8820,7 +8825,7 @@
       </c>
       <c r="I124" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Blood_Falls</t>
+          <t>NSF / Wikipedia — Blood Falls, Taylor Glacier Antarctica (Kan Şelalesi): https://en.wikipedia.org/wiki/Blood_Falls</t>
         </is>
       </c>
     </row>
@@ -8843,8 +8848,9 @@
       <c r="D125" s="14" t="inlineStr">
         <is>
           <t>Tam 5,5 milyon yıl boyunca güneş ışığının tek bir zerresini bile görmemiş, mühürlü bir yeraltı dünyasının kapısını açtığını hayal et. Romanya'da tesadüfen keşfedilen Movile Mağarası, dış dünyadan tamamen kopuk bambaşka bir gezegen gibi. İçerideki havada oksijen normalin yarısından bile az, atmosferi ise zehirli hidrojen sülfür ve karbondioksitle dolu. Güneş ışığı olmadığı için buradaki yaşam tamamen kimyasal enerjiyle ayakta kalıyor ve içeride gözleri yok olmuş, sadece buraya özgü 30'dan fazla gizemli canlı türü yaşıyor. Peki özel bir oksijen tüpüyle bu karanlık mağaraya inme şansın olsa içeri adım atar mıydın, yoksa kapısını mühürlü mü bırakırdın? Yorumlarda buluşalım!
-Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
-Kaynak: https://en.wikipedia.org/wiki/Movile_Cave
+💬 Peki özel bir oksijen tüpüyle bu karanlık mağaraya inme şansın olsa içeri adım atar mıydın, yoksa kapısını mühürlü mü bırakırdın? Yorumlarda buluşalım! 👇
+📚 Kaynak: BBC / Wikipedia — Movile Cave Chemosynthesis Ecosystem (Movile Mağarası): https://en.wikipedia.org/wiki/Movile_Cave
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #mağara #doğa #biyoloji #bilim</t>
         </is>
       </c>
@@ -8870,7 +8876,7 @@
       </c>
       <c r="I125" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Movile_Cave</t>
+          <t>BBC / Wikipedia — Movile Cave Chemosynthesis Ecosystem (Movile Mağarası): https://en.wikipedia.org/wiki/Movile_Cave</t>
         </is>
       </c>
     </row>
@@ -8893,8 +8899,9 @@
       <c r="D126" s="14" t="inlineStr">
         <is>
           <t>Şu gördüğün neon sarısı ve zümrüt yeşili göller başka bir gezegene değil, Dünya üzerindeki en tehlikeli cehenneme ait. Etiyopya'daki Danakil Çöküntüsü'nde yer alan Dallol Volkanı, deniz seviyesinin 48 metre altında kaynayan dev bir kimya laboratuvarı gibidir. Yerin altındaki kızgın magma, kalın tuz ve kükürt yataklarıyla buluştuğunda, yüzeye akü asidinden bile daha yakıcı kaynar sular ve zehirli klor gazları fışkırır. Burada maskesiz uzun süre nefes almak bile imkânsızdır. Peki sen uzaylı bir gezegeni andıran bu yeri uzaktan dronelarla izlemeyi mi seçerdin, yoksa özel koruyucu kıyafetle yanına kadar yürümeyi mi? Yorumlarda buluşalım!
-Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
-Kaynak: https://en.wikipedia.org/wiki/Dallol_(hydrothermal_system)
+💬 Peki sen uzaylı bir gezegeni andıran bu yeri uzaktan dronelarla izlemeyi mi seçerdin, yoksa özel koruyucu kıyafetle yanına kadar yürümeyi mi? Yorumlarda buluşalım! 👇
+📚 Kaynak: Nature Ecology &amp; Evolution / Wikipedia — Dallol Hydrothermal System: https://en.wikipedia.org/wiki/Dallol_(hydrothermal_system)
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #volkan #doğa #coğrafya #bilim</t>
         </is>
       </c>
@@ -8920,7 +8927,7 @@
       </c>
       <c r="I126" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Dallol_(hydrothermal_system)</t>
+          <t>Nature Ecology &amp; Evolution / Wikipedia — Dallol Hydrothermal System: https://en.wikipedia.org/wiki/Dallol_(hydrothermal_system)</t>
         </is>
       </c>
     </row>
@@ -8943,8 +8950,9 @@
       <c r="D127" s="14" t="inlineStr">
         <is>
           <t>Yerin tam 2.224 metre altına, yani üst üste dizilmiş 7 Eyfel Kulesi derinliğine karanlık bir kuyudan indiğini hayal et. Kafkas Dağları'ndaki Krubera Mağarası, Dünya'nın bilinen en derin uçurumlarından biridir. Buraya inen mağaracıların en dibe ulaşması haftalar sürer ve içeride yeraltı şelaleleriyle buz gibi su tünelleri vardır. En şaşırtıcı olanı ise, 2.000 metre derinlikteki o dondurucu ve ışıksız sularda bile dış dünyayı hiç görmemiş şeffaf canlıların yaşamaya devam etmesidir. Peki sana sınırsız ekipman verilse okyanusun en derin çukuruna dalmayı mı seçerdin, yoksa Dünya'nın en derin mağarasına inmeyi mi? Yorumlarda buluşalım!
-Daha fazla bilgi dozu için takip etmeyi unutma! 🔔
-Kaynak: https://en.wikipedia.org/wiki/Krubera_Cave
+💬 Peki sana sınırsız ekipman verilse okyanusun en derin çukuruna dalmayı mı seçerdin, yoksa Dünya'nın en derin mağarasına inmeyi mi? Yorumlarda buluşalım! 👇
+📚 Kaynak: National Geographic / Wikipedia — Krubera Cave (Dünya'nın En Derin Mağaraları): https://en.wikipedia.org/wiki/Krubera_Cave
+🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #mağara #doğa #keşif #bilim</t>
         </is>
       </c>
@@ -8970,7 +8978,7 @@
       </c>
       <c r="I127" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Krubera_Cave</t>
+          <t>National Geographic / Wikipedia — Krubera Cave (Dünya'nın En Derin Mağaraları): https://en.wikipedia.org/wiki/Krubera_Cave</t>
         </is>
       </c>
     </row>
@@ -8993,8 +9001,8 @@
       <c r="D128" s="14" t="inlineStr">
         <is>
           <t>Denizin dibinde iki bin yıl boyunca paslanmış bir Yunan batığından, modern saatler kadar karmaşık dişlilere sahip antik bir bilgisayar çıktığını biliyor muydun?
-Peki sence antik dünyada bunun gibi henüz keşfedemediğimiz başka yüksek teknolojiler de var mıdır, yoksa bu tek bir dahinin eseri miydi? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Antikythera_mechanism
+💬 Peki sence antik dünyada bunun gibi henüz keşfedemediğimiz başka yüksek teknolojiler de var mıdır, yoksa bu tek bir dahinin eseri miydi? Yorumlarda buluşalım! 👇
+📚 Kaynak: Nature / Wikipedia — Antikythera Mechanism (2.100 Yıllık Antik Analog Bilgisayar): https://en.wikipedia.org/wiki/Antikythera_mechanism
 🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #tarih #arkeoloji #bilim</t>
         </is>
@@ -9021,7 +9029,7 @@
       </c>
       <c r="I128" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Antikythera_mechanism</t>
+          <t>Nature / Wikipedia — Antikythera Mechanism (2.100 Yıllık Antik Analog Bilgisayar): https://en.wikipedia.org/wiki/Antikythera_mechanism</t>
         </is>
       </c>
     </row>
@@ -9044,8 +9052,8 @@
       <c r="D129" s="14" t="inlineStr">
         <is>
           <t>Kapadokya'nın altında, yirmi bin insanın hayvanları ve erzaklarıyla birlikte haftalarca hiç yeryüzüne çıkmadan yaşayabildiği sekiz katlı dev bir yeraltı şehri var: Derinkuyu.
-Peki sen tehlike anında haftalarca böyle bir yeraltı şehrinde yaşayabilir miydin, yoksa kapalı alanda daralır mıydın? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Derinkuyu_underground_city
+💬 Peki sen tehlike anında haftalarca böyle bir yeraltı şehrinde yaşayabilir miydin, yoksa kapalı alanda daralır mıydın? Yorumlarda buluşalım! 👇
+📚 Kaynak: UNESCO / Wikipedia — Derinkuyu Underground City (Derinkuyu Yeraltı Şehri): https://en.wikipedia.org/wiki/Derinkuyu_underground_city
 🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #tarih #arkeoloji #bilim</t>
         </is>
@@ -9072,7 +9080,7 @@
       </c>
       <c r="I129" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Derinkuyu_underground_city</t>
+          <t>UNESCO / Wikipedia — Derinkuyu Underground City (Derinkuyu Yeraltı Şehri): https://en.wikipedia.org/wiki/Derinkuyu_underground_city</t>
         </is>
       </c>
     </row>
@@ -9095,8 +9103,8 @@
       <c r="D130" s="14" t="inlineStr">
         <is>
           <t>Dünyanın en iyi şifre çözücüleri, dilbilimcileri ve yapay zekâları bir araya geldi ama altı yüz yıllık bu kitabın tek bir cümlesini bile okuyamadı: Voynich El Yazması.
-Peki sence bu kitap unutulmuş gizli bir bilimin şifreli kaydı mı, yoksa tarihin en zekice kurgulanmış bilmecesi mi? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Voynich_manuscript
+💬 Peki sence bu kitap unutulmuş gizli bir bilimin şifreli kaydı mı, yoksa tarihin en zekice kurgulanmış bilmecesi mi? Yorumlarda buluşalım! 👇
+📚 Kaynak: Yale Beinecke Library / Wikipedia — Voynich Manuscript (Voynich El Yazması): https://en.wikipedia.org/wiki/Voynich_manuscript
 🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #tarih #arkeoloji #bilim</t>
         </is>
@@ -9123,7 +9131,7 @@
       </c>
       <c r="I130" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Voynich_manuscript</t>
+          <t>Yale Beinecke Library / Wikipedia — Voynich Manuscript (Voynich El Yazması): https://en.wikipedia.org/wiki/Voynich_manuscript</t>
         </is>
       </c>
     </row>
@@ -9146,8 +9154,8 @@
       <c r="D131" s="14" t="inlineStr">
         <is>
           <t>Deniz seviyesinden üç bin sekiz yüz metre yüksekte, aralarına jilet bile girmeyecek kadar kusursuz kesilmiş yüz tonluk taş bloklar düşün: Puma Punku.
-Peki sence antik ustalar bu kusursuz taş işçiliğini sabırlı el aletleriyle mi başardı, yoksa bugün unuttuğumuz özel bir teknikleri mi vardı? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Pumapunku
+💬 Peki sence antik ustalar bu kusursuz taş işçiliğini sabırlı el aletleriyle mi başardı, yoksa bugün unuttuğumuz özel bir teknikleri mi vardı? Yorumlarda buluşalım! 👇
+📚 Kaynak: UNESCO / Wikipedia — Pumapunku Andesite Megaliths (Puma Punku H-Blokları): https://en.wikipedia.org/wiki/Pumapunku
 🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #tarih #arkeoloji #bilim</t>
         </is>
@@ -9174,7 +9182,7 @@
       </c>
       <c r="I131" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Pumapunku</t>
+          <t>UNESCO / Wikipedia — Pumapunku Andesite Megaliths (Puma Punku H-Blokları): https://en.wikipedia.org/wiki/Pumapunku</t>
         </is>
       </c>
     </row>
@@ -9197,8 +9205,8 @@
       <c r="D132" s="14" t="inlineStr">
         <is>
           <t>Dünyanın Yedi Harikası'ndan biri sayılan Babil'in Asma Bahçeleri'nin aslında hiçbir zaman Babil'de olmadığını duysan ne derdin?
-Peki sen geçmişe gidebilsen önce bu efsanevi Asma Bahçeleri'ni mi görmek isterdin, yoksa İskenderiye Kütüphanesi'ni mi? Yorumlarda buluşalım! 👇
-📚 Kaynak: https://en.wikipedia.org/wiki/Hanging_Gardens_of_Babylon
+💬 Peki sen geçmişe gidebilsen önce bu efsanevi Asma Bahçeleri'ni mi görmek isterdin, yoksa İskenderiye Kütüphanesi'ni mi? Yorumlarda buluşalım! 👇
+📚 Kaynak: Oxford University (Stephanie Dalley) / Wikipedia — Hanging Gardens of Babylon: https://en.wikipedia.org/wiki/Hanging_Gardens_of_Babylon
 🎨 Görseller temsilîdir (AI üretimi).
 #bilgidozu #shorts #tarih #arkeoloji #bilim</t>
         </is>
@@ -9225,7 +9233,7 @@
       </c>
       <c r="I132" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Hanging_Gardens_of_Babylon</t>
+          <t>Oxford University (Stephanie Dalley) / Wikipedia — Hanging Gardens of Babylon: https://en.wikipedia.org/wiki/Hanging_Gardens_of_Babylon</t>
         </is>
       </c>
     </row>
@@ -9282,9 +9290,9 @@
       </c>
       <c r="I133" s="14" t="inlineStr">
         <is>
-          <t>https://en.wikipedia.org/wiki/Bone_conduction
-https://en.wikipedia.org/wiki/The_imp_of_the_perverse
-https://en.wikipedia.org/wiki/Capsaicin</t>
+          <t>1) Kemik İletimi — Wikipedia: https://en.wikipedia.org/wiki/Bone_conduction
+2) Boşluğun Çağrısı — Wikipedia: https://en.wikipedia.org/wiki/The_imp_of_the_perverse
+3) Kapsaisin &amp; TRPV1 — Wikipedia: https://en.wikipedia.org/wiki/Capsaicin</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(sheets): mark video_35.mp4 (da3y0_DfWYQ) as YÜKLENDİ (A42:M42 Green)
</commit_message>
<xml_diff>
--- a/baslik.xlsx
+++ b/baslik.xlsx
@@ -3021,56 +3021,64 @@
       <c r="M41" s="4" t="inlineStr"/>
     </row>
     <row r="42" ht="42" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>YÜKLENMEDİ</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>YÜKLENDİ</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>video_35.mp4</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>Vücudundaki Tüm Acıyı Yöneten Beynin Kendisi Acı Hissedemez! 🧠⚡ #bilgidozu #shorts</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>Elimiz yandığında ya da dizimiz çarptığında acıyı bize hissettiren merkez beyindir; ancak beyin dokusunun kendisinde tek bir ağrı alıcısı (nosiseptör) bile yoktur! Baş ağrısı dediğimiz şey aslında beynin kendisinden değil, onu saran zarlar ve kan damarlarındaki gerilimden kaynaklanır.
 Daha fazla bilgi dozu için takip etmeyi unutma!</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
+      <c r="E42" s="3" t="inlineStr">
         <is>
           <t>#bilgidozu #shorts #beyin #bilim</t>
         </is>
       </c>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="F42" s="3" t="inlineStr">
         <is>
           <t>bilgidozu, beyin, ağrı, nörobilim, anatomi, insanvücudu, ilginçbilgiler, bilim, shorts</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G42" s="3" t="inlineStr">
         <is>
           <t>Beyin dokusunun hiç acı hissetmediğini biliyor muydun? 🧠⚡ Bilenler '1', yeni öğrenenler '2' yazsın! 👇</t>
         </is>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H42" s="4" t="inlineStr">
         <is>
           <t>Beyin ve Psikoloji</t>
         </is>
       </c>
-      <c r="I42" s="6" t="inlineStr">
+      <c r="I42" s="3" t="inlineStr">
         <is>
           <t>BrainFacts (Society for Neuroscience): https://www.brainfacts.org/</t>
         </is>
       </c>
-      <c r="J42" s="6" t="inlineStr"/>
-      <c r="K42" s="7" t="inlineStr"/>
-      <c r="L42" s="7" t="inlineStr"/>
-      <c r="M42" s="7" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>https://youtu.be/da3y0_DfWYQ</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-24 18:22</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr"/>
+      <c r="M42" s="4" t="inlineStr"/>
     </row>
     <row r="43" ht="42" customHeight="1">
       <c r="A43" s="5" t="inlineStr">
@@ -8107,7 +8115,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24 17:55</t>
+          <t>2026-10-24 18:22</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -8116,11 +8124,11 @@
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>video_34.mp4 yayınlandı (https://youtu.be/tCuQNw_V74I) · Sıradaki: video_35.mp4</t>
+          <t>video_35.mp4 yayınlandı (https://youtu.be/da3y0_DfWYQ) · Sıradaki: video_36.mp4</t>
         </is>
       </c>
     </row>
@@ -8456,7 +8464,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Sıradaki Shorts: video_35.mp4 · Sıradaki Uzun Video: uzun_video_8.mp4 yayın saatini bekliyor.</t>
+          <t>Sıradaki Shorts: video_36.mp4 · Sıradaki Uzun Video: uzun_video_8.mp4 yayın saatini bekliyor.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(queue): lock MIN_SHORTS_NUMBER=131 so only new approved series enters release
</commit_message>
<xml_diff>
--- a/baslik.xlsx
+++ b/baslik.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M134"/>
+  <dimension ref="A1:M135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -8100,6 +8100,56 @@
       <c r="L134" s="5" t="n"/>
       <c r="M134" s="5" t="n"/>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>BEKLEMEDE</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>video_131.mp4</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Kâğıt Kesiği Neden Bu Kadar Acıtır? 🩹 #bilgidozu #shorts</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Küçücük bir kâğıt kesiği neden beklediğinden çok daha fazla can yakar? Parmak uçlarımız dokunma ve ağrıyı algılayan yoğun duyu sinirleriyle donatılmıştır. Üstelik çıplak gözle düz görünen kâğıt kenarı, mikroskobik ölçekte lifli ve düzensiz bir yapıya sahiptir; gün boyu ellerimizi kullanmaya devam etmemiz de hassaslaşan dokuyu tekrar tekrar uyarır.
+Senin de başına geldi mi? Yorumlarda buluşalım! 👇
+📚 Kaynak: Dr. Hayley Goldbach (UCLA Dermatology) / BBC Future &amp; StatPearls
+🎨 Görseller temsilîdir (AI bilimsel canlandırma).</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>#bilgidozu #shorts #insanvücudu #beyin #bilim</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>bilgi dozu, kağıt kesiği, insan vücudu, duyu sinirleri, bilim, ilginç bilgiler, shorts</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Senin de başına geldi mi? En son ne zaman kâğıt kesiği yaşadın, yorumlara yaz! 👇</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>İnsan Vücudu ve Beyin</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>BBC Future (Dr. H. Goldbach, UCLA, 2016) &amp; StatPearls</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>